<commit_message>
transitioned to google api calls
</commit_message>
<xml_diff>
--- a/assets/temp.xlsx
+++ b/assets/temp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23426"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\avtopia\data_sync_desktop\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E85BFB0-4244-4BB2-A329-035970007BAE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD435383-ECC9-434E-B688-5DE109EEBA25}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21330" yWindow="0" windowWidth="20655" windowHeight="15600" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="1647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="1649">
   <si>
     <t>ID</t>
   </si>
@@ -197,7 +197,7 @@
     <t>Palm Beach Aircraft Service Inc.</t>
   </si>
   <si>
-    <t>2633 Lantana Rd </t>
+    <t>2633 Lantana Rd</t>
   </si>
   <si>
     <t>Suite 41</t>
@@ -863,7 +863,7 @@
     <t>Purvis Brothers Inc.</t>
   </si>
   <si>
-    <t>PO Box 957321 </t>
+    <t>PO Box 957321</t>
   </si>
   <si>
     <t>Mars Valencia Rd</t>
@@ -1721,7 +1721,7 @@
     <t>Shoals Flight Center/ NW Alabama Reg. Arprt</t>
   </si>
   <si>
-    <t>1729 T Ed Campbell Dr </t>
+    <t>1729 T Ed Campbell Dr</t>
   </si>
   <si>
     <t>Suite A</t>
@@ -1760,7 +1760,7 @@
     <t>Siam Land Flying</t>
   </si>
   <si>
-    <t>222 Don Mueang International Airport Office </t>
+    <t>222 Don Mueang International Airport Office</t>
   </si>
   <si>
     <t>Vibhavadi Rangsit Road Sanambin Don Mueang</t>
@@ -1904,7 +1904,7 @@
     <t>Sky Harbor Aviation</t>
   </si>
   <si>
-    <t>855 Saint Johns Bluff Rd N </t>
+    <t>855 Saint Johns Bluff Rd N</t>
   </si>
   <si>
     <t>Hangar 5</t>
@@ -3395,7 +3395,7 @@
     <t>Thro Avation (Zen Flight)</t>
   </si>
   <si>
-    <t>1000 New Highway </t>
+    <t>1000 New Highway</t>
   </si>
   <si>
     <t>Hangar #81</t>
@@ -3530,7 +3530,7 @@
     <t>Top Flight Detail</t>
   </si>
   <si>
-    <t>Mobile Regional Airport </t>
+    <t>Mobile Regional Airport</t>
   </si>
   <si>
     <t>371 Flave Pierce Road</t>
@@ -3764,7 +3764,7 @@
     <t>Tucson Aeroservice Center, Inc.</t>
   </si>
   <si>
-    <t>11700 W Avra Valley Rd </t>
+    <t>11700 W Avra Valley Rd</t>
   </si>
   <si>
     <t>Unit 85</t>
@@ -3905,7 +3905,7 @@
     <t>University of North Dakota, UND Aerospace Division</t>
   </si>
   <si>
-    <t>2798 Airport Dr </t>
+    <t>2798 Airport Dr</t>
   </si>
   <si>
     <t>Stop 9052</t>
@@ -4454,7 +4454,7 @@
     <t>West Houston Airport</t>
   </si>
   <si>
-    <t>PO Box 941789 </t>
+    <t>PO Box 941789</t>
   </si>
   <si>
     <t>18000 Groeschke Rd</t>
@@ -4970,16 +4970,22 @@
     <t>Google:Longitude</t>
   </si>
   <si>
-    <t>Executive Air</t>
+    <t>X</t>
+  </si>
+  <si>
+    <t>{"business_status":"OPERATIONAL","formatted_address":"2633 Lantana Rd #41, Lantana, FL 33462, USA","geometry":{"location":{"lat":26.5891232,"lng":-80.085217},"viewport":{"northeast":{"lat":26.5903062802915,"lng":-80.08379641970849},"southwest":{"lat":26.5876083197085,"lng":-80.0864943802915}}},"icon":"https://maps.gstatic.com/mapfiles/place_api/icons/v1/png_71/generic_business-71.png","name":"Palm Beach Aircraft Services Inc","place_id":"ChIJ4S0GlInY2IgRuTZrggV5fA0","plus_code":{"compound_code":"HWQ7+JW Lantana, FL, USA","global_code":"76RXHWQ7+JW"},"types":["point_of_interest","establishment"]}</t>
+  </si>
+  <si>
+    <t>Palm Beach Aircraft Services Inc</t>
   </si>
   <si>
     <t>OPERATIONAL</t>
   </si>
   <si>
-    <t>ChIJ43oI8gD5AogRU3iIWdpibqI</t>
-  </si>
-  <si>
-    <t>2131 Airport Dr, Green Bay, WI 54313, USA</t>
+    <t>ChIJ4S0GlInY2IgRuTZrggV5fA0</t>
+  </si>
+  <si>
+    <t>2633 Lantana Rd #41, Lantana, FL 33462, USA</t>
   </si>
 </sst>
 </file>
@@ -14307,7 +14313,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{478346B4-F175-45F8-959F-E74CD3C87AD8}">
-  <dimension ref="A1:Y263"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="10.875" style="3"/>
@@ -14325,7 +14331,7 @@
     <col min="14" max="14" width="23.875" style="3" customWidth="1"/>
     <col min="15" max="15" width="23.875" style="3" bestFit="1" customWidth="1"/>
     <col min="16" max="18" width="23.875" style="3" customWidth="1"/>
-    <col min="19" max="19" width="11.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="255.625" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="16384" width="10.875" style="3"/>
   </cols>
   <sheetData>
@@ -14431,24 +14437,6 @@
       <c r="L2" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="T2" t="s">
-        <v>1643</v>
-      </c>
-      <c r="U2" t="s">
-        <v>1644</v>
-      </c>
-      <c r="V2" t="s">
-        <v>1645</v>
-      </c>
-      <c r="W2" t="s">
-        <v>1646</v>
-      </c>
-      <c r="X2">
-        <v>44.4936934</v>
-      </c>
-      <c r="Y2">
-        <v>-88.1296081</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -14478,23 +14466,29 @@
       <c r="L3" s="5" t="s">
         <v>57</v>
       </c>
+      <c r="O3" t="s">
+        <v>1643</v>
+      </c>
+      <c r="S3" s="22" t="s">
+        <v>1644</v>
+      </c>
       <c r="T3" t="s">
-        <v>1643</v>
+        <v>1645</v>
       </c>
       <c r="U3" t="s">
-        <v>1644</v>
+        <v>1646</v>
       </c>
       <c r="V3" t="s">
-        <v>1645</v>
+        <v>1647</v>
       </c>
       <c r="W3" t="s">
-        <v>1646</v>
+        <v>1648</v>
       </c>
       <c r="X3">
-        <v>44.4936934</v>
+        <v>26.5891232</v>
       </c>
       <c r="Y3">
-        <v>-88.1296081</v>
+        <v>-80.085217</v>
       </c>
     </row>
     <row r="4">
@@ -14525,24 +14519,6 @@
       <c r="M4" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="T4" t="s">
-        <v>1643</v>
-      </c>
-      <c r="U4" t="s">
-        <v>1644</v>
-      </c>
-      <c r="V4" t="s">
-        <v>1645</v>
-      </c>
-      <c r="W4" t="s">
-        <v>1646</v>
-      </c>
-      <c r="X4">
-        <v>44.4936934</v>
-      </c>
-      <c r="Y4">
-        <v>-88.1296081</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -14572,24 +14548,6 @@
       <c r="M5" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="T5" t="s">
-        <v>1643</v>
-      </c>
-      <c r="U5" t="s">
-        <v>1644</v>
-      </c>
-      <c r="V5" t="s">
-        <v>1645</v>
-      </c>
-      <c r="W5" t="s">
-        <v>1646</v>
-      </c>
-      <c r="X5">
-        <v>44.4936934</v>
-      </c>
-      <c r="Y5">
-        <v>-88.1296081</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -14615,24 +14573,6 @@
       </c>
       <c r="L6" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="T6" t="s">
-        <v>1643</v>
-      </c>
-      <c r="U6" t="s">
-        <v>1644</v>
-      </c>
-      <c r="V6" t="s">
-        <v>1645</v>
-      </c>
-      <c r="W6" t="s">
-        <v>1646</v>
-      </c>
-      <c r="X6">
-        <v>44.4936934</v>
-      </c>
-      <c r="Y6">
-        <v>-88.1296081</v>
       </c>
     </row>
   </sheetData>

</xml_diff>